<commit_message>
Remoção de arquivos não utilizados, duplicatas de componentes e exibição de placa de video na tela builds
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_ordens_pendentes.xlsx
+++ b/relatorios/relatorio_ordens_pendentes.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>ID Pedido</t>
   </si>
@@ -30,6 +30,15 @@
   </si>
   <si>
     <t>Status Ordem</t>
+  </si>
+  <si>
+    <t>Teste</t>
+  </si>
+  <si>
+    <t>2026-06-11</t>
+  </si>
+  <si>
+    <t>PENDENTE (0 dias)</t>
   </si>
 </sst>
 </file>
@@ -98,14 +107,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="8.87109375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="6.69140625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.9765625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="9.9609375" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="12.20703125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="10.4375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="15.85546875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -125,6 +134,23 @@
         <v>4</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D2" t="n" s="2">
+        <v>3027.0</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>